<commit_message>
docs(revision-note): record 2026-09-21 against the commits it describes
Release Summary and Engineering Log carry one Unreleased row for the
preflight tool, the trigger-gate work and the illumination
precondition, with the four commit hashes as evidence.

Four Validation Evidence rows, and the fourth is NOT RECORDED on
purpose: the illumination precondition and stable_frames 6 -> 3 both
still need a live line start. The three that passed were measured
locally, with no CI run for these commits yet, and the row says so
rather than letting a green full-suite stand in for field validation.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/yolo_inference_RevisionNote.xlsx
+++ b/docs/yolo_inference_RevisionNote.xlsx
@@ -1498,7 +1498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D27"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="16.2"/>
   <cols>
     <col width="15" customWidth="1" style="27" min="1" max="1"/>
@@ -1978,6 +1978,26 @@
       <c r="D27" s="29" t="inlineStr">
         <is>
           <t>Recorded crash-safe inspection release, rollback, and retention; fail-closed scoped pilot, preflight, and duplicate evidence; live-station test isolation; exact-SHA CI; and the Cable1/A report_only safety default. Verdicts remain fail-closed, but persisted triage-reason mapping is still incomplete for count/position configuration lookup and no-detection color cases. This is an integration entry, not a formal package or production certification.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="108" customHeight="1" s="41">
+      <c r="A28" s="60" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B28" s="29" t="inlineStr">
+        <is>
+          <t>Unreleased</t>
+        </is>
+      </c>
+      <c r="C28" s="29" t="inlineStr">
+        <is>
+          <t>Deployment Preflight, Trigger Latency, and an Illumination Precondition</t>
+        </is>
+      </c>
+      <c r="D28" s="29" t="inlineStr">
+        <is>
+          <t>Added tools/system_check, a standalone preflight that answers whether a Windows machine can run this application and how fast it does, with every threshold traceable to a file in the repository and the unstated ones named as unstated. Removed a camera frame that the auto-trigger state machine spent on a state change alone and retuned Cable1/A's gate: 480 ms median end-to-end on 2026-09-10 against 345 ms on 2026-09-21. Added a fifth golden-sample precondition so a pre-shift colour check cannot run while illumination is still outside its luma band and then report the result as a colour deviation.</t>
         </is>
       </c>
     </row>
@@ -2000,7 +2020,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.2"/>
   <cols>
     <col width="13" customWidth="1" style="41" min="1" max="1"/>
@@ -3103,6 +3123,61 @@
         </is>
       </c>
       <c r="I25" s="47" t="inlineStr">
+        <is>
+          <t>Dio Wang</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="268" customHeight="1" s="41">
+      <c r="A26" s="61" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B26" s="46" t="inlineStr">
+        <is>
+          <t>Unreleased</t>
+        </is>
+      </c>
+      <c r="C26" s="47" t="inlineStr">
+        <is>
+          <t>Three gaps found while preparing a second station. (1) No way to tell whether a target machine could run the application before installing it; requirements were spread across pins, configs, and code paths with no statement of which are real. (2) Auto-trigger latency was ~500 ms and PRODUCT_APPEAR consumed a whole camera frame without scoring anything. (3) Illumination auto-calibration logs and gives up when it cannot converge, but nothing stopped the golden-sample check from then running at the wrong brightness and reporting a colour deviation at a position.</t>
+        </is>
+      </c>
+      <c r="D26" s="47" t="inlineStr">
+        <is>
+          <t>Core changes
+- Added tools/system_check: OS/CPU/memory/disk/GPU/dependency/runtime/camera/network checks plus a benchmark of the real ONNX path, txt + JSON reports, and baseline comparison with per-metric direction.
+- Packaged-build package versions read from _internal metadata instead of by import; absence of a pure-Python package in a bundle reported as UNKNOWN, not missing.
+- PRODUCT_APPEAR now scores the frame on which it enters WAIT_STABLE.
+- Cable1/A auto_trigger.yaml: appear_frames 3-&gt;2, stable_frames 6-&gt;3, inspection_cooldown_ms 500-&gt;250; calibrated product_area_threshold preserved.
+- Illumination calibration outcome recorded; fifth readiness precondition (照明已收斂) reads it without I/O.
+Reverted
+- OpenCL letterbox: 24 ms in a microbenchmark, no improvement and ~3 ms slower against 82 production records. The benchmark's 'realistic conditions' did not mirror the real call order.</t>
+        </is>
+      </c>
+      <c r="E26" s="47" t="inlineStr">
+        <is>
+          <t>tools/system_check/** (27 files); tests/test_system_check_{checks,benchmark,report}.py
+core/auto_trigger.py; models/Cable1/A/auto_trigger.yaml; tests/test_auto_trigger_latency.py
+app/gui/auto_calibration_handler.py; app/gui/color_preflight_handler.py; tests/test_golden_sample_illumination_gate.py
+CHANGELOG.md; docs/DOCUMENTATION_INDEX.md; .gitignore</t>
+        </is>
+      </c>
+      <c r="F26" s="47" t="inlineStr">
+        <is>
+          <t>2026-09-21 local regression: 2388 passed, 6 skipped (full suite, Python 3.10.18, yolo_anomalib). ruff clean including the CI correctness gate over core app camera tools tests; mypy clean on new modules, unchanged error counts on the two touched GUI files. Standalone executable rebuilt from a clean venv (193 MB) and smoke tested with PATH reduced to System32 against both a source checkout and a packaged build: exit 0, no failures. Trigger latency measured from the application log: 480 ms median (n=23, 2026-09-10) against 345 ms (n=16, 2026-09-21). Per-inspection inference_time from Result/inspection_records.sqlite3: 57.0 ms median before, 60.0 ms after -- which is what reverted the OpenCL change.</t>
+        </is>
+      </c>
+      <c r="G26" s="47" t="inlineStr">
+        <is>
+          <t>The illumination precondition has not been exercised against a real line start; the failure it prevents was reproduced from recorded state. stable_frames 6-&gt;3 has not been validated on production boards -- the risk is a blurred capture, and FAIL rate and annotated-image sharpness are still to be watched. tools/system_check has no CI job. The benchmark's default synthetic frame yields one detection against six expected, so its postprocess figure is a lower bound. The target station's camera remains unverified (yolo11_inference.exe --check-camera-grab), and the packaged artifact still carries kornia 0.6.9 against a pinned 0.8.1 because the build environment is behind requirements.txt.</t>
+        </is>
+      </c>
+      <c r="H26" s="47" t="inlineStr">
+        <is>
+          <t>Inference: 14043f2, cc2376a, e1ae111, 393cee5</t>
+        </is>
+      </c>
+      <c r="I26" s="47" t="inlineStr">
         <is>
           <t>Dio Wang</t>
         </is>
@@ -3126,7 +3201,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.2"/>
   <cols>
     <col width="13" customWidth="1" style="41" min="1" max="1"/>
@@ -3805,6 +3880,202 @@
         </is>
       </c>
     </row>
+    <row r="17" ht="88" customHeight="1" s="41">
+      <c r="A17" s="59" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B17" s="47" t="inlineStr">
+        <is>
+          <t>yolo11_inference</t>
+        </is>
+      </c>
+      <c r="C17" s="47" t="inlineStr">
+        <is>
+          <t>3.10.18</t>
+        </is>
+      </c>
+      <c r="D17" s="47" t="inlineStr">
+        <is>
+          <t>2.4.1+cpu</t>
+        </is>
+      </c>
+      <c r="E17" s="47" t="inlineStr">
+        <is>
+          <t>yolo_anomalib</t>
+        </is>
+      </c>
+      <c r="F17" s="47" t="inlineStr">
+        <is>
+          <t>pytest</t>
+        </is>
+      </c>
+      <c r="G17" s="47" t="inlineStr">
+        <is>
+          <t>Full suite after preflight tool, trigger-gate and illumination-precondition changes</t>
+        </is>
+      </c>
+      <c r="H17" s="49" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I17" s="47" t="inlineStr">
+        <is>
+          <t>2388 passed, 6 skipped</t>
+        </is>
+      </c>
+      <c r="J17" s="47" t="inlineStr">
+        <is>
+          <t>Local run on the development station; no CI run for these commits yet. ruff (incl. CI correctness gate) and mypy clean.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="88" customHeight="1" s="41">
+      <c r="A18" s="59" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B18" s="47" t="inlineStr">
+        <is>
+          <t>yolo11_inference</t>
+        </is>
+      </c>
+      <c r="C18" s="47" t="inlineStr">
+        <is>
+          <t>3.11.9</t>
+        </is>
+      </c>
+      <c r="D18" s="47" t="inlineStr">
+        <is>
+          <t>not bundled</t>
+        </is>
+      </c>
+      <c r="E18" s="47" t="inlineStr">
+        <is>
+          <t>clean venv (onnxruntime, numpy, opencv-python, PyYAML, psutil, pyinstaller)</t>
+        </is>
+      </c>
+      <c r="F18" s="47" t="inlineStr">
+        <is>
+          <t>PyInstaller + manual</t>
+        </is>
+      </c>
+      <c r="G18" s="47" t="inlineStr">
+        <is>
+          <t>Standalone preflight executable: build, then run with PATH reduced to System32 against a source checkout and a packaged build</t>
+        </is>
+      </c>
+      <c r="H18" s="49" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I18" s="47" t="inlineStr">
+        <is>
+          <t>exit 0, 0 FAIL</t>
+        </is>
+      </c>
+      <c r="J18" s="47" t="inlineStr">
+        <is>
+          <t>193 MB. Built from a fresh venv so no developer-machine state leaks in.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="88" customHeight="1" s="41">
+      <c r="A19" s="59" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B19" s="47" t="inlineStr">
+        <is>
+          <t>Integrated system</t>
+        </is>
+      </c>
+      <c r="C19" s="47" t="inlineStr">
+        <is>
+          <t>3.10.18</t>
+        </is>
+      </c>
+      <c r="D19" s="47" t="inlineStr">
+        <is>
+          <t>2.4.1+cpu</t>
+        </is>
+      </c>
+      <c r="E19" s="47" t="inlineStr">
+        <is>
+          <t>Production station</t>
+        </is>
+      </c>
+      <c r="F19" s="47" t="inlineStr">
+        <is>
+          <t>Field measurement</t>
+        </is>
+      </c>
+      <c r="G19" s="47" t="inlineStr">
+        <is>
+          <t>Auto-trigger end-to-end latency; per-inspection inference_time</t>
+        </is>
+      </c>
+      <c r="H19" s="49" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="I19" s="47" t="inlineStr">
+        <is>
+          <t>480 -&gt; 345 ms median</t>
+        </is>
+      </c>
+      <c r="J19" s="47" t="inlineStr">
+        <is>
+          <t>From detection_20260910.log (n=23) and detection_20260921.log (n=16), and 96 inspection records. Camera grab verified on the development station only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="88" customHeight="1" s="41">
+      <c r="A20" s="59" t="n">
+        <v>46286</v>
+      </c>
+      <c r="B20" s="47" t="inlineStr">
+        <is>
+          <t>Integrated system</t>
+        </is>
+      </c>
+      <c r="C20" s="47" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D20" s="47" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="E20" s="47" t="inlineStr">
+        <is>
+          <t>Production station</t>
+        </is>
+      </c>
+      <c r="F20" s="47" t="inlineStr">
+        <is>
+          <t>Field validation</t>
+        </is>
+      </c>
+      <c r="G20" s="47" t="inlineStr">
+        <is>
+          <t>Golden-sample illumination precondition; stable_frames 6-&gt;3 on real boards</t>
+        </is>
+      </c>
+      <c r="H20" s="49" t="inlineStr">
+        <is>
+          <t>NOT RECORDED</t>
+        </is>
+      </c>
+      <c r="I20" s="47" t="inlineStr"/>
+      <c r="J20" s="47" t="inlineStr">
+        <is>
+          <t>Both still require a live line start. The precondition was reproduced from recorded calibration state, not from a real startup.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A4:J16"/>
   <mergeCells count="2">

</xml_diff>